<commit_message>
fix: complète le short de Procedure.code avec les terminologies à utiliser
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com> e8fa99353ec85a541bf7dc1244086a0842beee0b
</commit_message>
<xml_diff>
--- a/nr-doc-core-procedure/ig/StructureDefinition-fr-core-procedure.xlsx
+++ b/nr-doc-core-procedure/ig/StructureDefinition-fr-core-procedure.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-09-16T15:10:32+00:00</t>
+    <t>2026-09-16T15:30:48+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -752,7 +752,7 @@
 </t>
   </si>
   <si>
-    <t>Code d'acte</t>
+    <t>Code d'acte : CCAM (facturante), SNOMED CT (international, additional binding) ou CISIS 'Autre acte'/absent-unknown</t>
   </si>
   <si>
     <t>Identification of the procedure or recording of "absence of relevant procedures" or of "procedures unknown".</t>

</xml_diff>